<commit_message>
added names to shifts
</commit_message>
<xml_diff>
--- a/frontend/public/schedule_template.xlsx
+++ b/frontend/public/schedule_template.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Employees" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Availability" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Shifts" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Availability" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shifts" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -826,7 +826,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr"/>
@@ -967,14 +967,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -985,20 +986,25 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Shift Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Start Time</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>End Time</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Required Skills</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Min Staff</t>
         </is>
@@ -1012,20 +1018,25 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>Optional label, e.g. Morning Shift (shown on the chart instead of the times)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
           <t>HH:MM (24-hour)</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>HH:MM (24-hour)</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Comma-separated skills required (leave blank for any employee)</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>How many staff needed for this shift (default 1)</t>
         </is>
@@ -1034,525 +1045,630 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
+          <t>Morning Shift</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
           <t>08:00</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="D3" s="10" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="D3" s="10" t="inlineStr">
+      <c r="E3" s="10" t="inlineStr">
         <is>
           <t>cashier, first_aid</t>
         </is>
       </c>
-      <c r="E3" s="10" t="n">
+      <c r="F3" s="10" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
+          <t>Morning Shift</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
           <t>08:00</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="D4" s="11" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="E4" s="11" t="inlineStr">
         <is>
           <t>cashier</t>
         </is>
       </c>
-      <c r="E4" s="11" t="n">
+      <c r="F4" s="11" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
+          <t>Evening Shift</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="D5" s="10" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="E5" s="10" t="inlineStr">
         <is>
           <t>cashier</t>
         </is>
       </c>
-      <c r="E5" s="10" t="n">
+      <c r="F5" s="10" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
+          <t>Morning Shift</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
           <t>08:00</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="D6" s="11" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>cashier, first_aid</t>
         </is>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="F6" s="11" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
+          <t>Morning Shift</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
           <t>08:00</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="E7" s="10" t="inlineStr">
         <is>
           <t>cashier</t>
         </is>
       </c>
-      <c r="E7" s="10" t="n">
+      <c r="F7" s="10" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
+          <t>Evening Shift</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="D8" s="11" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="D8" s="11" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>cashier</t>
         </is>
       </c>
-      <c r="E8" s="11" t="n">
+      <c r="F8" s="11" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
+          <t>Morning Shift</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
           <t>08:00</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>cashier, first_aid</t>
         </is>
       </c>
-      <c r="E9" s="10" t="n">
+      <c r="F9" s="10" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
+          <t>Morning Shift</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
           <t>08:00</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="D10" s="11" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="D10" s="11" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>cashier</t>
         </is>
       </c>
-      <c r="E10" s="11" t="n">
+      <c r="F10" s="11" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
+          <t>Evening Shift</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="D11" s="10" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="E11" s="10" t="inlineStr">
         <is>
           <t>cashier</t>
         </is>
       </c>
-      <c r="E11" s="10" t="n">
+      <c r="F11" s="10" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
+          <t>Morning Shift</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
           <t>08:00</t>
         </is>
       </c>
-      <c r="C12" s="11" t="inlineStr">
+      <c r="D12" s="11" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="D12" s="11" t="inlineStr">
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>cashier, first_aid</t>
         </is>
       </c>
-      <c r="E12" s="11" t="n">
+      <c r="F12" s="11" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
+          <t>Morning Shift</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
           <t>08:00</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr">
+      <c r="D13" s="10" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="D13" s="10" t="inlineStr">
+      <c r="E13" s="10" t="inlineStr">
         <is>
           <t>cashier</t>
         </is>
       </c>
-      <c r="E13" s="10" t="n">
+      <c r="F13" s="10" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
+          <t>Evening Shift</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
+      <c r="D14" s="11" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="D14" s="11" t="inlineStr">
+      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>cashier</t>
         </is>
       </c>
-      <c r="E14" s="11" t="n">
+      <c r="F14" s="11" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
+          <t>Morning Shift</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
           <t>08:00</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="D15" s="10" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="D15" s="10" t="inlineStr">
+      <c r="E15" s="10" t="inlineStr">
         <is>
           <t>cashier, first_aid</t>
         </is>
       </c>
-      <c r="E15" s="10" t="n">
+      <c r="F15" s="10" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
+          <t>Morning Shift</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
           <t>08:00</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="D16" s="11" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="D16" s="11" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>cashier</t>
         </is>
       </c>
-      <c r="E16" s="11" t="n">
+      <c r="F16" s="11" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
+          <t>Evening Shift</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C17" s="10" t="inlineStr">
+      <c r="D17" s="10" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="D17" s="10" t="inlineStr">
+      <c r="E17" s="10" t="inlineStr">
         <is>
           <t>cashier</t>
         </is>
       </c>
-      <c r="E17" s="10" t="n">
+      <c r="F17" s="10" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
+          <t>Morning Shift</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
           <t>08:00</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="D18" s="11" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>cashier, first_aid</t>
         </is>
       </c>
-      <c r="E18" s="11" t="n">
+      <c r="F18" s="11" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
+          <t>Morning Shift</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
           <t>08:00</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr">
+      <c r="D19" s="10" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="D19" s="10" t="inlineStr">
+      <c r="E19" s="10" t="inlineStr">
         <is>
           <t>cashier</t>
         </is>
       </c>
-      <c r="E19" s="10" t="n">
+      <c r="F19" s="10" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
+          <t>Evening Shift</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
+      <c r="D20" s="11" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="D20" s="11" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>cashier</t>
         </is>
       </c>
-      <c r="E20" s="11" t="n">
+      <c r="F20" s="11" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
+          <t>Morning Shift</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
           <t>08:00</t>
         </is>
       </c>
-      <c r="C21" s="10" t="inlineStr">
+      <c r="D21" s="10" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="D21" s="10" t="inlineStr">
+      <c r="E21" s="10" t="inlineStr">
         <is>
           <t>cashier, first_aid</t>
         </is>
       </c>
-      <c r="E21" s="10" t="n">
+      <c r="F21" s="10" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
+          <t>Morning Shift</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
           <t>08:00</t>
         </is>
       </c>
-      <c r="C22" s="11" t="inlineStr">
+      <c r="D22" s="11" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="D22" s="11" t="inlineStr">
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>cashier</t>
         </is>
       </c>
-      <c r="E22" s="11" t="n">
+      <c r="F22" s="11" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
+          <t>Evening Shift</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C23" s="10" t="inlineStr">
+      <c r="D23" s="10" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="D23" s="10" t="inlineStr">
+      <c r="E23" s="10" t="inlineStr">
         <is>
           <t>cashier</t>
         </is>
       </c>
-      <c r="E23" s="10" t="n">
+      <c r="F23" s="10" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>